<commit_message>
Record independent packaging removal acceptance and migration backups
</commit_message>
<xml_diff>
--- a/docs/templates/期初盘点模板-简化版.xlsx
+++ b/docs/templates/期初盘点模板-简化版.xlsx
@@ -5482,25 +5482,24 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J5001"/>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="C2:C5001">
       <formula1>SKU编号列表</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="D2:D5001" operator="between">
-      <formula1>0</formula1>
-      <formula2>9223372036854775807</formula2>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="A2:A5001">
+      <formula1>OR(C2="",COUNTIFS($A$2:$A$5001,A2,$C$2:$C$5001,C2)=1)</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="F2:F5001" operator="between">
-      <formula1>0</formula1>
-      <formula2>9223372036854775807</formula2>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="D2:D5001">
+      <formula1>AND(ISNUMBER(D2),D2=INT(D2),D2&gt;=0,SUM($F2:$G2,$I2)&lt;=$D2)</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="G2:G5001" operator="between">
-      <formula1>0</formula1>
-      <formula2>9223372036854775807</formula2>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="F2:F5001">
+      <formula1>AND(ISNUMBER(F2),F2=INT(F2),F2&gt;=0,SUM($F2:$G2,$I2)&lt;=$D2)</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="I2:I5001" operator="between">
-      <formula1>0</formula1>
-      <formula2>9223372036854775807</formula2>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="G2:G5001">
+      <formula1>AND(ISNUMBER(G2),G2=INT(G2),G2&gt;=0,SUM($F2:$G2,$I2)&lt;=$D2)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="I2:I5001">
+      <formula1>AND(ISNUMBER(I2),I2=INT(I2),I2&gt;=0,SUM($F2:$G2,$I2)&lt;=$D2)</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="请检查填写内容" error="请按模板规则填写，导入时仍会再次校验。" sqref="E2:E5001">
       <formula1>AND(ISNUMBER(E2),E2&gt;=0,E2=ROUND(E2,3))</formula1>

</xml_diff>